<commit_message>
feat: add 5th room type (Presidential Silk Suite) and enrich room images with captions
</commit_message>
<xml_diff>
--- a/mock-data/mock_hotel_database.xlsx
+++ b/mock-data/mock_hotel_database.xlsx
@@ -897,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>https://images.unsplash.com/photo-1618773928121-c32242e63f39?auto=format&amp;fit=crop&amp;w=800&amp;q=80</t>
+          <t>Không gian phòng ngủ Cozy (Bedroom view) (https://images.unsplash.com/photo-1618773928121-c32242e63f39?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bàn làm việc và góc đọc sách (Workspace view) (https://images.unsplash.com/photo-1505691938895-1758d7feb511?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng tắm đứng hiện đại (Bathroom view) (https://images.unsplash.com/photo-1552321554-5fecd8c7856a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Lối vào và tủ quần áo (Entrance view) (https://images.unsplash.com/photo-1540518614846-7eded433c457?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>https://images.unsplash.com/photo-1590490360182-c33d57733427?auto=format&amp;fit=crop&amp;w=800&amp;q=80</t>
+          <t>Giường ngủ đôi King Size sang trọng (Bedroom view) (https://images.unsplash.com/photo-1590490360182-c33d57733427?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bồn tắm nằm cao cấp (Bathtub view) (https://images.unsplash.com/photo-1584622650111-993a426fbf0a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Ban công và cửa sổ ngắm phố cổ (Balcony &amp; City view) (https://images.unsplash.com/photo-1600585154340-be6161a56a0c?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Không gian chi tiết trong phòng (Interior detail) (https://images.unsplash.com/photo-1591088398332-8a7791972843?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Quầy Mini-bar và máy pha cà phê (Mini-bar &amp; Coffee setup) (https://images.unsplash.com/photo-1565008447742-97f6f38c985c?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>https://images.unsplash.com/photo-1566665797739-1674de7a421a?auto=format&amp;fit=crop&amp;w=800&amp;q=80</t>
+          <t>Giường ngủ Super King và phòng ngủ (Bedroom view) (https://images.unsplash.com/photo-1566665797739-1674de7a421a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng khách sang trọng riêng biệt (Living room view) (https://images.unsplash.com/photo-1582719508461-905c673771fd?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bồn tắm Jacuzzi sục khí mát-xa (Jacuzzi view) (https://images.unsplash.com/photo-1507038772120-7bef2c68207a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Tầm nhìn từ ban công hướng thẳng Hồ Gươm (Lake View from balcony) (https://images.unsplash.com/photo-1513694203232-719a280e022f?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Giỏ trái cây tươi và dịch vụ chào đón (Welcome amenities) (https://images.unsplash.com/photo-1512918728675-ed5a9ecdebfd?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -1196,12 +1196,69 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>https://images.unsplash.com/photo-1578683010236-d716f9a3f461?auto=format&amp;fit=crop&amp;w=800&amp;q=80</t>
+          <t>Phòng ngủ lớn kết nối cửa thông (Connecting Master room) (https://images.unsplash.com/photo-1578683010236-d716f9a3f461?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng ngủ 2 giường đơn cho các con (Twin Bed room) (https://images.unsplash.com/photo-1568495248636-6432b97bd949?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng tắm gia đình tiện nghi (Family bathroom view) (https://images.unsplash.com/photo-1600566753190-17f0baa2a6c3?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Khu vực góc nghỉ ngơi chung cho gia đình (Sofa corner) (https://images.unsplash.com/photo-1502672260266-1c1ef2d93688?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Chi tiết đồ amenities cho trẻ nhỏ (Kids set) (https://images.unsplash.com/photo-1616594039964-ae9021a400a0?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Hạng phòng tối ưu nhất cho nhóm gia đình 4-6 người. Do số lượng phòng Connecting hạn chế, vui lòng liên hệ xác nhận trước.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>room_005</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Presidential Silk Suite</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Căn hộ Tổng thống đỉnh cao của sự sang trọng, kết hợp thiết kế hoàng gia Pháp - Đông Dương và các dịch vụ đặc quyền riêng.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>2 Giường đôi cỡ Super King ở 2 phòng ngủ riêng biệt</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Toàn cảnh 360 độ Hồ Hoàn Kiếm, Tháp Rùa và Phố Cổ Hà Nội từ tầng cao nhất</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>• Hai phòng ngủ khép kín với phòng tắm riêng biệt
+• Phòng khách và phòng ăn lớn sang trọng có quầy Bar riêng
+• Ban công siêu rộng với bồn tắm sục Jacuzzi ngoài trời nhìn ra Hồ Gươm
+• Phòng xông hơi hơi nước riêng (Steam Room)
+• Dịch vụ quản gia phục vụ 24/7
+• Đầu bếp phục vụ món ăn tại phòng theo thực đơn riêng
+• Đưa đón sân bay khứ hồi bằng xe hạng sang (Limousine Dcar) miễn phí</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Phòng ngủ Tổng thống thượng hạng (Presidential Bedroom) (https://images.unsplash.com/photo-1631049307264-da0ec9d70304?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng khách hoàng gia rộng lớn (Royal Living room) (https://images.unsplash.com/photo-1600210492486-724fe5c67fb0?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bể sục Jacuzzi ngoài trời trên ban công lớn (Outdoor Jacuzzi &amp; View) (https://images.unsplash.com/photo-1571896349842-33c89424de2d?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng tắm lát đá cẩm thạch và phòng xông hơi (Marble Bathroom &amp; Sauna) (https://images.unsplash.com/photo-1600607687920-4e2a09cf159d?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng ăn riêng và quầy Bar cá nhân (Private Dining &amp; Bar) (https://images.unsplash.com/photo-1600566752355-35792bedcfea?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Trải nghiệm lưu trú cao cấp bậc nhất tại Hà Nội. Yêu cầu đặt trước 72 giờ và thanh toán đặt cọc 100%.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: replace broken unsplash image links with working ones
</commit_message>
<xml_diff>
--- a/mock-data/mock_hotel_database.xlsx
+++ b/mock-data/mock_hotel_database.xlsx
@@ -1019,7 +1019,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Không gian phòng ngủ Cozy (Bedroom view) (https://images.unsplash.com/photo-1618773928121-c32242e63f39?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bàn làm việc và góc đọc sách (Workspace view) (https://images.unsplash.com/photo-1505691938895-1758d7feb511?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng tắm đứng hiện đại (Bathroom view) (https://images.unsplash.com/photo-1552321554-5fecd8c7856a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Lối vào và tủ quần áo (Entrance view) (https://images.unsplash.com/photo-1540518614846-7eded433c457?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
+          <t>Không gian phòng ngủ Cozy (Bedroom view) (https://images.unsplash.com/photo-1618773928121-c32242e63f39?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bàn làm việc và góc đọc sách (Workspace view) (https://images.unsplash.com/photo-1505691938895-1758d7feb511?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng tắm đứng hiện đại (Bathroom view) (https://images.unsplash.com/photo-1584622781564-1d987f7333c1?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Lối vào và tủ quần áo (Entrance view) (https://images.unsplash.com/photo-1540518614846-7eded433c457?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Giường ngủ Super King và phòng ngủ (Bedroom view) (https://images.unsplash.com/photo-1566665797739-1674de7a421a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng khách sang trọng riêng biệt (Living room view) (https://images.unsplash.com/photo-1582719508461-905c673771fd?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bồn tắm Jacuzzi sục khí mát-xa (Jacuzzi view) (https://images.unsplash.com/photo-1507038772120-7bef2c68207a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Tầm nhìn từ ban công hướng thẳng Hồ Gươm (Lake View from balcony) (https://images.unsplash.com/photo-1513694203232-719a280e022f?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Giỏ trái cây tươi và dịch vụ chào đón (Welcome amenities) (https://images.unsplash.com/photo-1512918728675-ed5a9ecdebfd?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
+          <t>Giường ngủ Super King và phòng ngủ (Bedroom view) (https://images.unsplash.com/photo-1566665797739-1674de7a421a?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Phòng khách sang trọng riêng biệt (Living room view) (https://images.unsplash.com/photo-1582719508461-905c673771fd?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Bồn tắm Jacuzzi sục khí mát-xa (Jacuzzi view) (https://images.unsplash.com/photo-1600607687939-ce8a6c25118c?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Tầm nhìn từ ban công hướng thẳng Hồ Gươm (Lake View from balcony) (https://images.unsplash.com/photo-1513694203232-719a280e022f?auto=format&amp;fit=crop&amp;w=800&amp;q=80); Giỏ trái cây tươi và dịch vụ chào đón (Welcome amenities) (https://images.unsplash.com/photo-1512918728675-ed5a9ecdebfd?auto=format&amp;fit=crop&amp;w=800&amp;q=80)</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">

</xml_diff>